<commit_message>
Changes to the Component Selection
</commit_message>
<xml_diff>
--- a/docs/06-Power-Budget/Christo-power-budget.xlsx
+++ b/docs/06-Power-Budget/Christo-power-budget.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81AA136B-3B70-4B12-B671-D500212A6C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA104E3-E340-43F3-A51C-A4C78A1E0543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Budget" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Power Budget'!$A$1:$H$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Power Budget'!$A$1:$H$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="41">
   <si>
     <t>Christo Power Budget</t>
   </si>
@@ -73,9 +73,6 @@
   </si>
   <si>
     <t>Version:</t>
-  </si>
-  <si>
-    <t>1.0</t>
   </si>
   <si>
     <t>A. List ALL major components (active devices, integrated circuits, etc.) except for power sources, voltage regulators, resistors, capacitors, or passive elements</t>
@@ -182,6 +179,15 @@
   </si>
   <si>
     <t>Private use Door automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microcontroller </t>
+  </si>
+  <si>
+    <t>PIC18F57Q43 CURIOSITY NANO</t>
+  </si>
+  <si>
+    <t>+1.7 - 5.1 V</t>
   </si>
 </sst>
 </file>
@@ -386,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -414,33 +420,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -455,11 +439,32 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -810,8 +815,8 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
-  <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H73"/>
+  <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="22.5" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.125" style="1" customWidth="1"/>
@@ -824,19 +829,19 @@
     <col min="10" max="16384" width="13.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -846,12 +851,12 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="2"/>
@@ -860,12 +865,12 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
@@ -874,12 +879,12 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>5</v>
+      <c r="B5" s="7">
+        <v>2</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="2"/>
@@ -888,7 +893,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -898,533 +903,580 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="31"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20"/>
-    </row>
-    <row r="8" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="B8" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="C8" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="D8" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="E8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="F8" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="G8" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="H8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="32" t="s">
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="8"/>
+      <c r="B9" s="16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="26" t="s">
+      <c r="C9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="D9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="E9" s="16">
+        <v>1</v>
+      </c>
+      <c r="F9" s="16">
+        <v>6</v>
+      </c>
+      <c r="G9" s="16">
+        <v>6</v>
+      </c>
+      <c r="H9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="26">
-        <v>1</v>
-      </c>
-      <c r="F9" s="26">
+    </row>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A10" s="8"/>
+      <c r="B10" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="16">
+        <v>1</v>
+      </c>
+      <c r="F10" s="16">
+        <v>10</v>
+      </c>
+      <c r="G10" s="16">
+        <v>10</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="8"/>
+      <c r="B11" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="16">
+        <v>1</v>
+      </c>
+      <c r="F11" s="16">
+        <v>1</v>
+      </c>
+      <c r="G11" s="16">
+        <v>1</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A12" s="8"/>
+      <c r="B12" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="16">
+        <v>1</v>
+      </c>
+      <c r="F12" s="16">
+        <v>20</v>
+      </c>
+      <c r="G12" s="16">
+        <v>20</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="36">
+        <v>1</v>
+      </c>
+      <c r="F13" s="36">
+        <v>500</v>
+      </c>
+      <c r="G13" s="37">
+        <v>500</v>
+      </c>
+      <c r="H13" s="37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A16" s="8"/>
+      <c r="B16" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="16">
         <v>6</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G16" s="16">
         <v>6</v>
       </c>
-      <c r="H9" s="26" t="s">
+      <c r="H16" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A17" s="8"/>
+      <c r="B17" s="16" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="26" t="s">
+      <c r="C17" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="D17" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="16">
+        <v>1</v>
+      </c>
+      <c r="F17" s="16">
+        <v>10</v>
+      </c>
+      <c r="G17" s="16">
+        <v>10</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A18" s="8"/>
+      <c r="B18" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="C18" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="16">
+        <v>1</v>
+      </c>
+      <c r="F18" s="16">
+        <v>1</v>
+      </c>
+      <c r="G18" s="16">
+        <v>1</v>
+      </c>
+      <c r="H18" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="26">
-        <v>1</v>
-      </c>
-      <c r="F10" s="26">
-        <v>10</v>
-      </c>
-      <c r="G10" s="26">
-        <v>10</v>
-      </c>
-      <c r="H10" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="26" t="s">
+    </row>
+    <row r="19" spans="1:8" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="39"/>
+      <c r="B19" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="36">
+        <v>1</v>
+      </c>
+      <c r="F19" s="36">
+        <v>500</v>
+      </c>
+      <c r="G19" s="37">
+        <v>500</v>
+      </c>
+      <c r="H19" s="37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="13"/>
+      <c r="B20" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="C20" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="23">
+        <v>1</v>
+      </c>
+      <c r="F20" s="23">
+        <v>20</v>
+      </c>
+      <c r="G20" s="23">
+        <v>20</v>
+      </c>
+      <c r="H20" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="26">
-        <v>1</v>
-      </c>
-      <c r="F11" s="26">
-        <v>1</v>
-      </c>
-      <c r="G11" s="26">
-        <v>1</v>
-      </c>
-      <c r="H11" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="26">
-        <v>1</v>
-      </c>
-      <c r="F12" s="26">
-        <v>20</v>
-      </c>
-      <c r="G12" s="26">
-        <v>20</v>
-      </c>
-      <c r="H12" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-    </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="34" t="s">
+    </row>
+    <row r="21" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+    </row>
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D22" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="32" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="26" t="s">
+      <c r="E22" s="33"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="16">
+        <f>SUM(G16:G21)</f>
+        <v>537</v>
+      </c>
+      <c r="H22" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D23" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="18">
+        <v>0.25</v>
+      </c>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D24" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="15"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="8">
+        <f>G22*1.25</f>
+        <v>671.25</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+    </row>
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="26" t="s">
+      <c r="D26" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" s="16">
+        <v>1</v>
+      </c>
+      <c r="F26" s="16">
+        <v>1500</v>
+      </c>
+      <c r="G26" s="16">
+        <v>1500</v>
+      </c>
+      <c r="H26" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="26">
-        <v>1</v>
-      </c>
-      <c r="F15" s="26">
-        <v>6</v>
-      </c>
-      <c r="G15" s="26">
-        <v>6</v>
-      </c>
-      <c r="H15" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="26" t="s">
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="23">
+        <f>G26-G24</f>
+        <v>828.75</v>
+      </c>
+      <c r="H27" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="26">
-        <v>1</v>
-      </c>
-      <c r="F16" s="26">
-        <v>10</v>
-      </c>
-      <c r="G16" s="26">
-        <v>10</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="26">
-        <v>1</v>
-      </c>
-      <c r="F17" s="26">
-        <v>1</v>
-      </c>
-      <c r="G17" s="26">
-        <v>1</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="35" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="35">
-        <v>1</v>
-      </c>
-      <c r="F18" s="35">
-        <v>20</v>
-      </c>
-      <c r="G18" s="35">
-        <v>20</v>
-      </c>
-      <c r="H18" s="35" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" s="21" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-    </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="28"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="26">
-        <f>SUM(G15:G19)</f>
-        <v>37</v>
-      </c>
-      <c r="H20" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="28"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="30">
-        <v>0.25</v>
-      </c>
-      <c r="H21" s="9"/>
-    </row>
-    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="25"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="8">
-        <f>G20*1.25</f>
-        <v>46.25</v>
-      </c>
-      <c r="H22" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-    </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="26">
-        <v>1</v>
-      </c>
-      <c r="F24" s="26">
-        <v>1500</v>
-      </c>
-      <c r="G24" s="26">
-        <v>1500</v>
-      </c>
-      <c r="H24" s="26" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="35">
-        <f>G24-G22</f>
-        <v>1453.75</v>
-      </c>
-      <c r="H25" s="35" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
-    </row>
-    <row r="32" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="17"/>
-    </row>
-    <row r="33" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="17"/>
-    </row>
-    <row r="34" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="36" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="17"/>
-    </row>
-    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="17"/>
-    </row>
-    <row r="42" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="17"/>
-    </row>
-    <row r="43" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="17"/>
-    </row>
-    <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="2:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="17"/>
-    </row>
-    <row r="47" spans="2:6" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="2:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="16"/>
-    </row>
-    <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="16"/>
-    </row>
-    <row r="53" spans="1:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="16"/>
-    </row>
-    <row r="54" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="16"/>
-      <c r="B54" s="16"/>
-      <c r="C54" s="16"/>
-      <c r="D54" s="16"/>
-      <c r="E54" s="16"/>
-      <c r="F54" s="17"/>
-    </row>
-    <row r="55" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="56" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="16"/>
-    </row>
-    <row r="60" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="16"/>
-    </row>
-    <row r="61" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="16"/>
-    </row>
-    <row r="62" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="16"/>
-      <c r="C62" s="16"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="16"/>
-      <c r="F62" s="17"/>
-    </row>
-    <row r="63" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="16"/>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="17"/>
-    </row>
-    <row r="65" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="67" spans="1:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="68" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="69" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="16"/>
-      <c r="B69" s="16"/>
-      <c r="C69" s="16"/>
-      <c r="D69" s="16"/>
-      <c r="E69" s="16"/>
-      <c r="F69" s="17"/>
-    </row>
-    <row r="70" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="16"/>
-      <c r="B70" s="16"/>
-      <c r="C70" s="16"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="16"/>
-      <c r="F70" s="17"/>
-      <c r="G70" s="17"/>
-      <c r="H70" s="17"/>
-    </row>
-    <row r="71" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="16"/>
-      <c r="B71" s="16"/>
-      <c r="C71" s="16"/>
-      <c r="D71" s="16"/>
-      <c r="E71" s="16"/>
-      <c r="F71" s="17"/>
-      <c r="G71" s="17"/>
-      <c r="H71" s="17"/>
+    </row>
+    <row r="28" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5"/>
+    <row r="29" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="32" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="33" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="25"/>
+    </row>
+    <row r="34" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="25"/>
+    </row>
+    <row r="35" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="25"/>
+    </row>
+    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="37" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="38" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="25"/>
+    </row>
+    <row r="39" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="40" spans="2:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="41" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="42" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="43" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="25"/>
+    </row>
+    <row r="44" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="25"/>
+    </row>
+    <row r="45" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="25"/>
+    </row>
+    <row r="46" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="47" spans="2:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="48" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B48" s="24"/>
+      <c r="C48" s="24"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="25"/>
+    </row>
+    <row r="49" spans="1:6" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="50" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A53" s="24"/>
+    </row>
+    <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A54" s="24"/>
+    </row>
+    <row r="55" spans="1:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="24"/>
+    </row>
+    <row r="56" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="24"/>
+      <c r="B56" s="24"/>
+      <c r="C56" s="24"/>
+      <c r="D56" s="24"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="25"/>
+    </row>
+    <row r="57" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="58" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="59" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="60" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="61" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A61" s="24"/>
+    </row>
+    <row r="62" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A62" s="24"/>
+    </row>
+    <row r="63" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="24"/>
+    </row>
+    <row r="64" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B64" s="24"/>
+      <c r="C64" s="24"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="25"/>
+    </row>
+    <row r="65" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="66" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A66" s="24"/>
+      <c r="B66" s="24"/>
+      <c r="C66" s="24"/>
+      <c r="D66" s="24"/>
+      <c r="E66" s="24"/>
+      <c r="F66" s="25"/>
+    </row>
+    <row r="67" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="68" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="69" spans="1:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="70" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="71" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A71" s="24"/>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="24"/>
+      <c r="F71" s="25"/>
+    </row>
+    <row r="72" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A72" s="24"/>
+      <c r="B72" s="24"/>
+      <c r="C72" s="24"/>
+      <c r="D72" s="24"/>
+      <c r="E72" s="24"/>
+      <c r="F72" s="25"/>
+      <c r="G72" s="25"/>
+      <c r="H72" s="25"/>
+    </row>
+    <row r="73" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A73" s="24"/>
+      <c r="B73" s="24"/>
+      <c r="C73" s="24"/>
+      <c r="D73" s="24"/>
+      <c r="E73" s="24"/>
+      <c r="F73" s="25"/>
+      <c r="G73" s="25"/>
+      <c r="H73" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="D33:F33"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A70:H70"/>
-    <mergeCell ref="A71:H71"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="A64:F64"/>
-    <mergeCell ref="A69:F69"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A53:A55"/>
+    <mergeCell ref="A61:A63"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="D43:F43"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="D35:F35"/>
   </mergeCells>
-  <conditionalFormatting sqref="G25:G26 G36:G37 G46">
+  <conditionalFormatting sqref="G27:G28 G38:G39 G48">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -1433,8 +1485,8 @@
   <pageMargins left="0.25" right="0" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="25" max="7" man="1"/>
-    <brk id="46" max="7" man="1"/>
+    <brk id="27" max="7" man="1"/>
+    <brk id="48" max="7" man="1"/>
   </rowBreaks>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated the Power Budget
</commit_message>
<xml_diff>
--- a/docs/06-Power-Budget/Christo-power-budget.xlsx
+++ b/docs/06-Power-Budget/Christo-power-budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA104E3-E340-43F3-A51C-A4C78A1E0543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92612D19-2BA2-4B8F-8E5E-CEEFE70051B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Power Budget" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Power Budget'!$A$1:$H$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Power Budget'!$A$1:$H$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="54">
   <si>
     <t>Christo Power Budget</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>Rotary Encoder</t>
-  </si>
-  <si>
-    <t>PEC11R-4215F-S0024</t>
   </si>
   <si>
     <t>Setup Button</t>
@@ -188,6 +185,48 @@
   </si>
   <si>
     <t>+1.7 - 5.1 V</t>
+  </si>
+  <si>
+    <t>External Power Source</t>
+  </si>
+  <si>
+    <t>Power Source 1 selection</t>
+  </si>
+  <si>
+    <t>WSU090-2000-R</t>
+  </si>
+  <si>
+    <t>9V 2A Power Supply</t>
+  </si>
+  <si>
+    <t>Output Voltage</t>
+  </si>
+  <si>
+    <t>9V</t>
+  </si>
+  <si>
+    <t>Power Rails Connected to External Power Source</t>
+  </si>
+  <si>
+    <t>+5V Voltage Regulator</t>
+  </si>
+  <si>
+    <t>LM7805</t>
+  </si>
+  <si>
+    <t>+5 - 35V</t>
+  </si>
+  <si>
+    <t>+110-220V</t>
+  </si>
+  <si>
+    <t>EM14R0D-R20-L064S</t>
+  </si>
+  <si>
+    <t>+1.8 - 5.5 V</t>
+  </si>
+  <si>
+    <t>5V</t>
   </si>
 </sst>
 </file>
@@ -392,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -439,16 +478,14 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -460,11 +497,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -815,14 +862,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="22.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="43.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.125" style="1" customWidth="1"/>
     <col min="3" max="3" width="27.5" style="1" customWidth="1"/>
     <col min="4" max="4" width="31" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.8125" style="1" customWidth="1"/>
     <col min="6" max="6" width="34.5" style="4" customWidth="1"/>
     <col min="7" max="8" width="18.5" style="4" customWidth="1"/>
     <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
@@ -830,16 +877,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="5" t="s">
@@ -856,7 +903,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="2"/>
@@ -870,7 +917,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
@@ -971,7 +1018,7 @@
         <v>18</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>16</v>
@@ -980,10 +1027,10 @@
         <v>1</v>
       </c>
       <c r="F10" s="16">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G10" s="16">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>17</v>
@@ -992,10 +1039,10 @@
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="8"/>
       <c r="B11" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>20</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>21</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>16</v>
@@ -1016,13 +1063,13 @@
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="8"/>
       <c r="B12" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="D12" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E12" s="16">
         <v>1</v>
@@ -1037,26 +1084,26 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B13" s="36" t="s">
+    <row r="13" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="36" t="s">
+      <c r="D13" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="36">
+      <c r="E13" s="14">
         <v>1</v>
       </c>
-      <c r="F13" s="36">
+      <c r="F13" s="14">
         <v>500</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="24">
         <v>500</v>
       </c>
-      <c r="H13" s="37" t="s">
+      <c r="H13" s="24" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1072,7 +1119,7 @@
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="20" t="s">
         <v>7</v>
@@ -1081,28 +1128,28 @@
         <v>8</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" s="20" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="21" t="s">
         <v>34</v>
-      </c>
-      <c r="G15" s="21" t="s">
-        <v>35</v>
       </c>
       <c r="H15" s="20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="8"/>
       <c r="B16" s="16" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>16</v>
@@ -1111,10 +1158,10 @@
         <v>1</v>
       </c>
       <c r="F16" s="16">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="G16" s="16">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="H16" s="16" t="s">
         <v>17</v>
@@ -1123,10 +1170,10 @@
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="8"/>
       <c r="B17" s="16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>16</v>
@@ -1135,95 +1182,85 @@
         <v>1</v>
       </c>
       <c r="F17" s="16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G17" s="16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H17" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="8"/>
-      <c r="B18" s="16" t="s">
+    <row r="18" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A18" s="26"/>
+      <c r="B18" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="14">
+        <v>1</v>
+      </c>
+      <c r="F18" s="14">
+        <v>500</v>
+      </c>
+      <c r="G18" s="24">
+        <v>500</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="13"/>
+      <c r="B19" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="23">
+        <v>1</v>
+      </c>
+      <c r="F19" s="23">
         <v>20</v>
       </c>
-      <c r="C18" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="16">
-        <v>1</v>
-      </c>
-      <c r="F18" s="16">
-        <v>1</v>
-      </c>
-      <c r="G18" s="16">
-        <v>1</v>
-      </c>
-      <c r="H18" s="16" t="s">
+      <c r="G19" s="23">
+        <v>20</v>
+      </c>
+      <c r="H19" s="23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="39"/>
-      <c r="B19" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="36">
-        <v>1</v>
-      </c>
-      <c r="F19" s="36">
-        <v>500</v>
-      </c>
-      <c r="G19" s="37">
-        <v>500</v>
-      </c>
-      <c r="H19" s="37" t="s">
+    <row r="20" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+    </row>
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D21" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="33"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="16">
+        <f>SUM(G16:G20)</f>
+        <v>547</v>
+      </c>
+      <c r="H21" s="16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="13"/>
-      <c r="B20" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="23">
-        <v>1</v>
-      </c>
-      <c r="F20" s="23">
-        <v>20</v>
-      </c>
-      <c r="G20" s="23">
-        <v>20</v>
-      </c>
-      <c r="H20" s="23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="D22" s="33" t="s">
@@ -1231,252 +1268,313 @@
       </c>
       <c r="E22" s="33"/>
       <c r="F22" s="34"/>
-      <c r="G22" s="16">
-        <f>SUM(G16:G21)</f>
-        <v>537</v>
-      </c>
-      <c r="H22" s="16" t="s">
+      <c r="G22" s="18">
+        <v>0.25</v>
+      </c>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D23" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="8">
+        <f>G21*1.25</f>
+        <v>683.75</v>
+      </c>
+      <c r="H23" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="D23" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="18">
-        <v>0.25</v>
-      </c>
-      <c r="H23" s="9"/>
-    </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="D24" s="15" t="s">
+    <row r="24" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A25" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="8">
-        <f>G22*1.25</f>
-        <v>671.25</v>
-      </c>
-      <c r="H24" s="16" t="s">
+      <c r="B25" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="16">
+        <v>1</v>
+      </c>
+      <c r="F25" s="16">
+        <v>1500</v>
+      </c>
+      <c r="G25" s="16">
+        <v>1500</v>
+      </c>
+      <c r="H25" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-    </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" s="16" t="s">
+    <row r="26" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="16">
-        <v>1</v>
-      </c>
-      <c r="F26" s="16">
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="23">
+        <f>G25-G23</f>
+        <v>816.25</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5"/>
+    <row r="28" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A28" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="F28" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="H28" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A29" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D29" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="16">
+        <v>2000</v>
+      </c>
+      <c r="G29" s="16">
+        <v>2000</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A30" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F30" s="9">
         <v>1500</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G30" s="9">
         <v>1500</v>
       </c>
-      <c r="H26" s="16" t="s">
+      <c r="H30" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B27" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="23">
-        <f>G26-G24</f>
-        <v>828.75</v>
-      </c>
-      <c r="H27" s="23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5"/>
-    <row r="29" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="32" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="33" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="25"/>
-    </row>
-    <row r="34" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="25"/>
-    </row>
-    <row r="35" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="25"/>
-    </row>
-    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="37" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="38" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="25"/>
-    </row>
-    <row r="39" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="40" spans="2:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="41" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="42" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="43" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="25"/>
-    </row>
-    <row r="44" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="25"/>
-    </row>
-    <row r="45" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="25"/>
-    </row>
-    <row r="46" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="47" spans="2:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="48" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="25"/>
-    </row>
-    <row r="49" spans="1:6" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="50" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="32" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="29"/>
+    </row>
+    <row r="33" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="29"/>
+    </row>
+    <row r="34" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="29"/>
+    </row>
+    <row r="35" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="36" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="37" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="29"/>
+    </row>
+    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="39" spans="2:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="40" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="41" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="42" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="29"/>
+    </row>
+    <row r="43" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="29"/>
+    </row>
+    <row r="44" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="29"/>
+    </row>
+    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="46" spans="2:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="47" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
+      <c r="F47" s="29"/>
+    </row>
+    <row r="48" spans="2:6" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="49" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A52" s="28"/>
+    </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A53" s="24"/>
-    </row>
-    <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A54" s="24"/>
-    </row>
-    <row r="55" spans="1:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="24"/>
-    </row>
-    <row r="56" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="24"/>
-      <c r="B56" s="24"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="25"/>
-    </row>
-    <row r="57" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="58" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+      <c r="A53" s="28"/>
+    </row>
+    <row r="54" spans="1:6" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="28"/>
+    </row>
+    <row r="55" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="28"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28"/>
+      <c r="F55" s="29"/>
+    </row>
+    <row r="56" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="57" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="58" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
     <row r="59" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="60" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="60" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A60" s="28"/>
+    </row>
     <row r="61" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A61" s="24"/>
-    </row>
-    <row r="62" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A62" s="24"/>
-    </row>
-    <row r="63" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="24"/>
-    </row>
-    <row r="64" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="25"/>
-    </row>
-    <row r="65" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="66" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="24"/>
-      <c r="B66" s="24"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="25"/>
-    </row>
-    <row r="67" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="68" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="69" spans="1:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="70" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+      <c r="A61" s="28"/>
+    </row>
+    <row r="62" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="28"/>
+    </row>
+    <row r="63" spans="1:6" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B63" s="28"/>
+      <c r="C63" s="28"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="28"/>
+      <c r="F63" s="29"/>
+    </row>
+    <row r="64" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="65" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A65" s="28"/>
+      <c r="B65" s="28"/>
+      <c r="C65" s="28"/>
+      <c r="D65" s="28"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="29"/>
+    </row>
+    <row r="66" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="67" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="68" spans="1:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="69" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="70" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A70" s="28"/>
+      <c r="B70" s="28"/>
+      <c r="C70" s="28"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="29"/>
+    </row>
     <row r="71" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A71" s="24"/>
-      <c r="B71" s="24"/>
-      <c r="C71" s="24"/>
-      <c r="D71" s="24"/>
-      <c r="E71" s="24"/>
-      <c r="F71" s="25"/>
-    </row>
-    <row r="72" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="24"/>
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="24"/>
-      <c r="F72" s="25"/>
-      <c r="G72" s="25"/>
-      <c r="H72" s="25"/>
-    </row>
-    <row r="73" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A73" s="24"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="24"/>
-      <c r="F73" s="25"/>
-      <c r="G73" s="25"/>
-      <c r="H73" s="25"/>
+      <c r="A71" s="28"/>
+      <c r="B71" s="28"/>
+      <c r="C71" s="28"/>
+      <c r="D71" s="28"/>
+      <c r="E71" s="28"/>
+      <c r="F71" s="29"/>
+      <c r="G71" s="29"/>
+      <c r="H71" s="29"/>
+    </row>
+    <row r="72" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A72" s="28"/>
+      <c r="B72" s="28"/>
+      <c r="C72" s="28"/>
+      <c r="D72" s="28"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="29"/>
+      <c r="G72" s="29"/>
+      <c r="H72" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="D34:F34"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A71:H71"/>
     <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A73:H73"/>
-    <mergeCell ref="A53:A55"/>
-    <mergeCell ref="A61:A63"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A52:A54"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="D42:F42"/>
     <mergeCell ref="D43:F43"/>
     <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="D21:F21"/>
     <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="D35:F35"/>
   </mergeCells>
-  <conditionalFormatting sqref="G27:G28 G38:G39 G48">
+  <conditionalFormatting sqref="G26:G27 G37:G38 G47">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -1485,8 +1583,8 @@
   <pageMargins left="0.25" right="0" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="27" max="7" man="1"/>
-    <brk id="48" max="7" man="1"/>
+    <brk id="26" max="7" man="1"/>
+    <brk id="47" max="7" man="1"/>
   </rowBreaks>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>